<commit_message>
Small wording changes in HW4 solution
</commit_message>
<xml_diff>
--- a/Homework 4/Homework 4 solution.xlsx
+++ b/Homework 4/Homework 4 solution.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
   <si>
     <t xml:space="preserve">Month</t>
   </si>
@@ -58,13 +58,13 @@
     <t xml:space="preserve">Value portfolio:</t>
   </si>
   <si>
-    <t xml:space="preserve">  alpha</t>
+    <t xml:space="preserve">  Alpha</t>
   </si>
   <si>
-    <t xml:space="preserve">  beta</t>
+    <t xml:space="preserve">  Beta</t>
   </si>
   <si>
-    <t xml:space="preserve">  sigma_e</t>
+    <t xml:space="preserve">  SD of regression residuals</t>
   </si>
   <si>
     <t xml:space="preserve">  IR</t>
@@ -73,13 +73,10 @@
     <t xml:space="preserve">Dollar-neutral:</t>
   </si>
   <si>
-    <t xml:space="preserve">(We calculated these numbers in class, so it’s also acceptable to just cite them.)</t>
-  </si>
-  <si>
     <t xml:space="preserve">We should assess active strategies based on IR.</t>
   </si>
   <si>
-    <t xml:space="preserve">So the investor would choose the long-only approach.</t>
+    <t xml:space="preserve">So the investor would choose the long-only approach, even though it has a lower alpha.</t>
   </si>
   <si>
     <t xml:space="preserve">Q2</t>
@@ -146,7 +143,7 @@
     <numFmt numFmtId="166" formatCode="yyyy\-mm"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -184,12 +181,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -241,7 +232,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -279,10 +270,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -418,9 +405,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="21.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="20.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="9.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="25.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="26.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="12.38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,9 +716,6 @@
       <c r="N8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="P8" s="2" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
@@ -931,7 +915,7 @@
         <v>-0.0039695</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -968,7 +952,7 @@
         <v>0.0223635</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1039,7 +1023,7 @@
         <v>-0.0160755</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1076,7 +1060,7 @@
         <v>0.0012285</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O17" s="1" t="n">
         <f aca="false">-INTERCEPT(D2:D361,B2:B361)</f>
@@ -1117,7 +1101,7 @@
         <v>-0.0269585</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1154,7 +1138,7 @@
         <v>-0.0247955</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1225,7 +1209,7 @@
         <v>0.045422</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1262,13 +1246,13 @@
         <v>0.004619</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O22" s="1" t="n">
         <f aca="false">CORREL(D2:D361,F2:F361)</f>
         <v>0.973875174511963</v>
       </c>
-      <c r="P22" s="10"/>
+      <c r="P22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="n">
@@ -1304,7 +1288,7 @@
         <v>0.0134195</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1375,7 +1359,7 @@
         <v>-0.021881</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1412,7 +1396,7 @@
         <v>0.0267895</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O26" s="1" t="n">
         <f aca="false">-INTERCEPT(F2:F361,B2:B361)</f>
@@ -1453,7 +1437,7 @@
         <v>0.0159685</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1524,7 +1508,7 @@
         <v>0.0541465</v>
       </c>
       <c r="N29" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1561,7 +1545,7 @@
         <v>0.00409399999999999</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O30" s="1" t="n">
         <f aca="false">-INTERCEPT(H2:H361,B2:B361)</f>
@@ -1602,7 +1586,7 @@
         <v>0.011983</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1803,7 +1787,7 @@
         <v>0.0387145</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1847,7 +1831,7 @@
         <v>0.00597908908307845</v>
       </c>
       <c r="P37" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1973,7 +1957,7 @@
         <v>0.220714767299246</v>
       </c>
       <c r="P40" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,7 +1994,7 @@
         <v>0.0085475</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2047,7 +2031,7 @@
         <v>-0.0202485</v>
       </c>
       <c r="N42" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>